<commit_message>
fixes made by dev and rerunning
</commit_message>
<xml_diff>
--- a/tests/TeamworkDB/output/utilization_failures_report_202606.xlsx
+++ b/tests/TeamworkDB/output/utilization_failures_report_202606.xlsx
@@ -592,15 +592,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -664,7 +664,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Officer</t>
+          <t>Manager</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -674,29 +674,29 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>1,073.30</t>
+          <t>1,890.00</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>1,107.10</t>
+          <t>2,067.20</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>33.80</t>
+          <t>177.20</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>3.15%</t>
+          <t>9.38%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>CRSV</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -711,222 +711,288 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>159.80</t>
+          <t>1,073.30</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>179.40</t>
+          <t>1,107.10</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>19.60</t>
+          <t>33.80</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>12.27%</t>
+          <t>3.15%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>CRCH</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Officer</t>
+          <t>Associate</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Standard_Rev</t>
+          <t>Actual_Hours</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>1,340,205.50</t>
+          <t>4,445.40</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>1,385,836.00</t>
+          <t>4,691.30</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>45,630.50</t>
+          <t>245.90</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>3.40%</t>
+          <t>5.53%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
+          <t>CRCH</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Actual_Hours</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>3,025.50</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>3,629.40</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>603.90</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>19.96%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>CRNY</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Actual_Hours</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>3,054.60</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>3,309.90</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>255.30</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>8.36%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
           <t>CRSV</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Actual_Hours</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>815.80</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>949.00</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>133.20</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>16.33%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>CRSV</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Officer</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>Standard_Rev</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>209,078.00</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>236,518.00</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>27,440.00</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>13.12%</t>
-        </is>
-      </c>
-    </row>
-    <row r="9"/>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Sheet: 2026_US (YTD)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Office</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Column</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>Util Report</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>DB</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>Diff</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>Diff%</t>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Actual_Hours</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>159.80</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>179.40</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>19.60</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>12.27%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>CRCH</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Officer</t>
+          <t>Analyst</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Actual_Hours</t>
+          <t>Standard_Rev</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>3,918.60</t>
+          <t>3,417,051.00</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>4,233.00</t>
+          <t>3,542,757.00</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>314.40</t>
+          <t>125,706.00</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>8.02%</t>
+          <t>3.68%</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>CRSF</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Analyst</t>
+          <t>Manager</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Actual_Hours</t>
+          <t>Standard_Rev</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>21,814.90</t>
+          <t>1,808,944.00</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>22,621.70</t>
+          <t>1,977,284.00</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>806.80</t>
+          <t>168,340.00</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>3.70%</t>
+          <t>9.31%</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>CRSV</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -936,27 +1002,27 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Actual_Hours</t>
+          <t>Standard_Rev</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>1,544.90</t>
+          <t>1,340,205.50</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>1,754.60</t>
+          <t>1,385,836.00</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>209.70</t>
+          <t>45,630.50</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>13.57%</t>
+          <t>3.40%</t>
         </is>
       </c>
     </row>
@@ -968,7 +1034,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Officer</t>
+          <t>Associate</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -978,34 +1044,34 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>5,000,596.50</t>
+          <t>3,348,962.00</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>5,456,477.00</t>
+          <t>3,514,945.00</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>455,880.50</t>
+          <t>165,983.00</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>9.12%</t>
+          <t>4.96%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>CRSF</t>
+          <t>CRCH</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Analyst</t>
+          <t>Manager</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -1015,57 +1081,953 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>11,191,272.50</t>
+          <t>2,978,296.00</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>11,657,616.00</t>
+          <t>3,543,916.00</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>466,343.50</t>
+          <t>565,620.00</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>4.17%</t>
+          <t>18.99%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
+          <t>CRNY</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Standard_Rev</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>2,975,824.50</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>3,211,977.00</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>236,152.50</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>7.94%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
           <t>CRSV</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Standard_Rev</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>787,357.00</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>913,897.00</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>126,540.00</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>16.07%</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>CRSV</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>Officer</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Standard_Rev</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>209,078.00</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>236,518.00</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>27,440.00</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>13.12%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Sheet: 2026_US (YTD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Column</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Util Report</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Diff</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Diff%</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Actual_Hours</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>9,949.60</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>10,882.80</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>933.20</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>9.38%</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>CRCH</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Associate</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Actual_Hours</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>24,679.55</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>25,782.90</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>1,103.35</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>4.47%</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>CRCH</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Actual_Hours</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>18,293.10</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>21,887.90</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>3,594.80</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>19.65%</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>CRCH</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Officer</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Actual_Hours</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>3,918.60</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>4,233.00</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>314.40</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>8.02%</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>CRDC</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Actual_Hours</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>21,469.10</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>22,583.50</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>1,114.40</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>5.19%</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>CRLA</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Analyst</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Actual_Hours</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>22,488.20</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>23,345.30</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>857.10</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>3.81%</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>CRLA</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Actual_Hours</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>8,326.70</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>9,104.90</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>778.20</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>9.35%</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>CRNY</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Actual_Hours</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>19,821.10</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>20,729.10</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>908.00</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>4.58%</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>CRSV</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Actual_Hours</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>5,050.10</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>5,931.90</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>881.80</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>17.46%</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>CRSV</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Officer</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Actual_Hours</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>1,544.90</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>1,754.60</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>209.70</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>13.57%</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Analyst</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Standard_Rev</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>20,194,754.00</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>20,804,404.00</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>609,650.00</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>3.02%</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Standard_Rev</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>9,619,478.50</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>10,506,019.00</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>886,540.50</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>9.22%</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>CRCH</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Associate</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Standard_Rev</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>18,607,382.25</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>19,348,397.00</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>741,014.75</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>3.98%</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>CRCH</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Standard_Rev</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>17,971,325.00</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>21,329,070.00</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>3,357,745.00</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>18.68%</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>CRCH</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Officer</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Standard_Rev</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>5,000,596.50</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>5,456,477.00</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>455,880.50</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>9.12%</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>CRDC</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Standard_Rev</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>21,080,120.00</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>22,110,940.00</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>1,030,820.00</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>4.89%</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>CRLA</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Analyst</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Standard_Rev</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>11,527,030.00</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>12,054,147.00</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>527,117.00</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>4.57%</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>CRLA</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Standard_Rev</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>8,003,047.50</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>8,742,338.00</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>739,290.50</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>9.24%</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>CRNY</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Standard_Rev</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>19,390,678.50</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>20,230,579.00</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>839,900.50</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>4.33%</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>CRSV</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Standard_Rev</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>4,878,389.00</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>5,716,099.00</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>837,710.00</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>17.17%</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>CRSV</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Officer</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Standard_Rev</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
         <is>
           <t>1,984,222.00</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E43" s="4" t="inlineStr">
         <is>
           <t>2,277,802.00</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F43" s="4" t="inlineStr">
         <is>
           <t>293,580.00</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G43" s="4" t="inlineStr">
         <is>
           <t>14.80%</t>
         </is>
@@ -1082,141 +2044,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>DB Employee Monthly</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Sheet: Month - CRCH (Monthly)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>EmpNo</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Column</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Util Report</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>DB</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Diff</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Diff%</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>101379</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Mahajan, Mansha</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Actual_Hours</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>132.50</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>161.90</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>29.40</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>22.19%</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>101379</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Mahajan, Mansha</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Standard_Rev</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>86,125.00</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>105,235.00</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>19,110.00</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>22.19%</t>
         </is>
       </c>
     </row>
@@ -1231,10 +2068,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1244,6 +2087,88 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Sheet: YTD - CRSF (YTD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>EmpNo</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Column</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Util Report</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Diff</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Diff%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>101650</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Li, Lily</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Actual_Hours</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>165.70</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>170.70</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>5.00</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>3.02%</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>